<commit_message>
Atualiza base de dados com novos Excel files (fA&B, ArenaKids, Estacionamento, Firezone)
Regenera data.js: 82 partidas, 1566 bordero rows, 3983 ingressos rows
KPIs: público total 1.610.092 · ticket médio R$ 31,41 · % sócios 62,6%

https://claude.ai/code/session_01QNVq88nQEVKfhevamvokrg
</commit_message>
<xml_diff>
--- a/fA&B.xlsx
+++ b/fA&B.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://safbotafogo-my.sharepoint.com/personal/pedro_arruda_safbfr_com_br/Documents/BI_2/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://safbotafogo-my.sharepoint.com/personal/pedro_arruda_safbfr_com_br/Documents/Área de Trabalho/dash-ticket/dash-ticket/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="68" documentId="8_{12E0946F-BA15-4933-9CDC-520F89AF3A34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{30F71DF4-31A7-4016-8A7E-C07B3E04BA97}"/>
+  <xr:revisionPtr revIDLastSave="88" documentId="8_{12E0946F-BA15-4933-9CDC-520F89AF3A34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9E46519A-EDF5-45D8-8788-14E32F00066C}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{41AE1BFD-0089-48BB-9F54-0C9C0739D654}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="69">
   <si>
     <t>2024.04.18-CAMBR2-2</t>
   </si>
@@ -216,6 +216,36 @@
   </si>
   <si>
     <t>2025.08.14-CAMLI5-OITAVAS</t>
+  </si>
+  <si>
+    <t>2026.01.21-CAMCA4-3</t>
+  </si>
+  <si>
+    <t>2026.01.24-CAMCA4-4</t>
+  </si>
+  <si>
+    <t>2026.01.29-CAMBR2-1</t>
+  </si>
+  <si>
+    <t>2026.02.01-CAMCA4-5</t>
+  </si>
+  <si>
+    <t>2026.02.15-CAMCA4-Quartas</t>
+  </si>
+  <si>
+    <t>2026.02.25-CAMLI5-2° FASE</t>
+  </si>
+  <si>
+    <t>2026.02.28-CAMCA4-SEMIS - TR</t>
+  </si>
+  <si>
+    <t>2026.03.07-CAMCA4-FINAL - TR</t>
+  </si>
+  <si>
+    <t>2026.03.10-CAMLI5-3° Fase</t>
+  </si>
+  <si>
+    <t>2026.03.14-CAMBR2-6</t>
   </si>
 </sst>
 </file>
@@ -607,12 +637,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC9C5773-1E3A-4441-BFAB-5B8FEBCDCDEA}">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:C93"/>
+  <dimension ref="A1:C103"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="25.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.36328125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -627,7 +656,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -638,7 +667,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -649,7 +678,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
@@ -660,7 +689,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
@@ -671,7 +700,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
@@ -682,7 +711,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
@@ -693,7 +722,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
@@ -704,7 +733,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
@@ -715,7 +744,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
@@ -726,7 +755,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
@@ -737,7 +766,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
@@ -748,7 +777,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>11</v>
       </c>
@@ -759,7 +788,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>12</v>
       </c>
@@ -770,7 +799,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="15" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>13</v>
       </c>
@@ -781,7 +810,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="16" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>14</v>
       </c>
@@ -792,7 +821,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>15</v>
       </c>
@@ -803,7 +832,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="18" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>16</v>
       </c>
@@ -825,7 +854,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="20" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>0</v>
       </c>
@@ -836,7 +865,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="21" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
         <v>1</v>
       </c>
@@ -847,7 +876,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="22" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>2</v>
       </c>
@@ -858,7 +887,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="23" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
         <v>3</v>
       </c>
@@ -869,7 +898,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>4</v>
       </c>
@@ -880,7 +909,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="25" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
         <v>5</v>
       </c>
@@ -891,7 +920,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="26" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>6</v>
       </c>
@@ -902,7 +931,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="27" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
         <v>7</v>
       </c>
@@ -913,7 +942,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="28" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>8</v>
       </c>
@@ -924,7 +953,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="29" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
         <v>9</v>
       </c>
@@ -935,7 +964,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="30" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>10</v>
       </c>
@@ -946,7 +975,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="31" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
         <v>11</v>
       </c>
@@ -957,7 +986,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="32" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
         <v>12</v>
       </c>
@@ -968,7 +997,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="33" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
         <v>13</v>
       </c>
@@ -979,7 +1008,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="34" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
         <v>14</v>
       </c>
@@ -990,7 +1019,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="35" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
         <v>15</v>
       </c>
@@ -1001,7 +1030,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="36" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
         <v>16</v>
       </c>
@@ -1023,7 +1052,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="38" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
         <v>23</v>
       </c>
@@ -1034,7 +1063,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="39" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
         <v>24</v>
       </c>
@@ -1045,7 +1074,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="40" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
         <v>25</v>
       </c>
@@ -1056,7 +1085,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="41" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
         <v>26</v>
       </c>
@@ -1067,7 +1096,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="42" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
         <v>27</v>
       </c>
@@ -1078,7 +1107,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="43" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
         <v>28</v>
       </c>
@@ -1089,7 +1118,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="44" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A44" s="2" t="s">
         <v>29</v>
       </c>
@@ -1100,7 +1129,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="45" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A45" s="2" t="s">
         <v>30</v>
       </c>
@@ -1111,7 +1140,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="46" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A46" s="2" t="s">
         <v>23</v>
       </c>
@@ -1122,7 +1151,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="47" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A47" s="2" t="s">
         <v>24</v>
       </c>
@@ -1133,7 +1162,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="48" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A48" s="2" t="s">
         <v>25</v>
       </c>
@@ -1144,7 +1173,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="49" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A49" s="2" t="s">
         <v>26</v>
       </c>
@@ -1155,7 +1184,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="50" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A50" s="2" t="s">
         <v>27</v>
       </c>
@@ -1166,7 +1195,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="51" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A51" s="2" t="s">
         <v>28</v>
       </c>
@@ -1177,7 +1206,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="52" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A52" s="2" t="s">
         <v>29</v>
       </c>
@@ -1188,7 +1217,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="53" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A53" s="2" t="s">
         <v>30</v>
       </c>
@@ -1199,7 +1228,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="54" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A54" s="2" t="s">
         <v>31</v>
       </c>
@@ -1210,7 +1239,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="55" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A55" s="2" t="s">
         <v>32</v>
       </c>
@@ -1221,7 +1250,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="56" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A56" s="2" t="s">
         <v>33</v>
       </c>
@@ -1232,7 +1261,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="57" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A57" s="2" t="s">
         <v>34</v>
       </c>
@@ -1243,7 +1272,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="58" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A58" s="2" t="s">
         <v>35</v>
       </c>
@@ -1254,7 +1283,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="59" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A59" s="2" t="s">
         <v>36</v>
       </c>
@@ -1265,7 +1294,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="60" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
         <v>37</v>
       </c>
@@ -1276,7 +1305,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="61" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A61" s="2" t="s">
         <v>31</v>
       </c>
@@ -1287,7 +1316,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="62" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A62" s="2" t="s">
         <v>32</v>
       </c>
@@ -1298,7 +1327,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="63" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A63" s="2" t="s">
         <v>33</v>
       </c>
@@ -1309,7 +1338,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="64" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A64" s="2" t="s">
         <v>34</v>
       </c>
@@ -1320,7 +1349,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="65" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A65" s="2" t="s">
         <v>35</v>
       </c>
@@ -1331,7 +1360,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="66" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A66" s="2" t="s">
         <v>36</v>
       </c>
@@ -1342,7 +1371,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="67" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A67" s="2" t="s">
         <v>37</v>
       </c>
@@ -1353,7 +1382,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="68" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A68" s="2" t="s">
         <v>38</v>
       </c>
@@ -1364,7 +1393,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="69" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A69" s="2" t="s">
         <v>39</v>
       </c>
@@ -1375,7 +1404,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="70" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A70" s="2" t="s">
         <v>40</v>
       </c>
@@ -1386,7 +1415,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="71" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A71" s="2" t="s">
         <v>41</v>
       </c>
@@ -1397,7 +1426,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="72" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A72" s="2" t="s">
         <v>42</v>
       </c>
@@ -1408,7 +1437,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="73" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A73" s="2" t="s">
         <v>38</v>
       </c>
@@ -1419,7 +1448,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="74" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A74" s="2" t="s">
         <v>39</v>
       </c>
@@ -1430,7 +1459,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="75" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A75" s="2" t="s">
         <v>40</v>
       </c>
@@ -1441,7 +1470,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="76" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A76" s="2" t="s">
         <v>41</v>
       </c>
@@ -1452,7 +1481,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="77" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A77" s="2" t="s">
         <v>42</v>
       </c>
@@ -1463,7 +1492,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="78" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A78" s="2" t="s">
         <v>43</v>
       </c>
@@ -1474,7 +1503,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="79" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A79" s="2" t="s">
         <v>44</v>
       </c>
@@ -1485,7 +1514,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="80" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A80" s="2" t="s">
         <v>45</v>
       </c>
@@ -1496,7 +1525,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="81" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A81" s="2" t="s">
         <v>46</v>
       </c>
@@ -1507,7 +1536,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="82" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A82" s="2" t="s">
         <v>47</v>
       </c>
@@ -1518,7 +1547,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="83" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A83" s="2" t="s">
         <v>48</v>
       </c>
@@ -1529,7 +1558,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="84" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A84" s="2" t="s">
         <v>49</v>
       </c>
@@ -1540,7 +1569,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="85" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A85" s="2" t="s">
         <v>50</v>
       </c>
@@ -1551,7 +1580,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="86" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A86" s="2" t="s">
         <v>51</v>
       </c>
@@ -1562,7 +1591,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="87" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A87" s="2" t="s">
         <v>52</v>
       </c>
@@ -1573,7 +1602,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="88" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A88" s="2" t="s">
         <v>53</v>
       </c>
@@ -1584,7 +1613,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="89" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A89" s="2" t="s">
         <v>54</v>
       </c>
@@ -1595,7 +1624,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="90" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A90" s="2" t="s">
         <v>55</v>
       </c>
@@ -1606,7 +1635,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="91" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A91" s="2" t="s">
         <v>56</v>
       </c>
@@ -1617,7 +1646,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="92" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A92" s="2" t="s">
         <v>57</v>
       </c>
@@ -1628,7 +1657,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="93" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A93" s="2" t="s">
         <v>58</v>
       </c>
@@ -1639,14 +1668,118 @@
         <v>21</v>
       </c>
     </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A94" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B94" s="3">
+        <v>23693.7</v>
+      </c>
+      <c r="C94" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A95" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B95" s="3">
+        <v>23862.2</v>
+      </c>
+      <c r="C95" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A96" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B96" s="3">
+        <v>76437.820000000007</v>
+      </c>
+      <c r="C96" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A97" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B97" s="3">
+        <v>47181.2</v>
+      </c>
+      <c r="C97" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A98" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B98" s="3">
+        <v>58570.5</v>
+      </c>
+      <c r="C98" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A99" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B99" s="3">
+        <v>118956.7</v>
+      </c>
+      <c r="C99" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A100" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B100" s="3">
+        <v>16904.3</v>
+      </c>
+      <c r="C100" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A101" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B101" s="3">
+        <v>32677</v>
+      </c>
+      <c r="C101" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A102" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B102" s="3">
+        <v>142680.70000000001</v>
+      </c>
+      <c r="C102" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A103" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B103" s="3">
+        <v>78269.399999999994</v>
+      </c>
+      <c r="C103" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C93" xr:uid="{DC9C5773-1E3A-4441-BFAB-5B8FEBCDCDEA}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="2024.12.08-CAMBR2-38"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:C93" xr:uid="{DC9C5773-1E3A-4441-BFAB-5B8FEBCDCDEA}"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
</xml_diff>